<commit_message>
Atualiza Lista de Jogos Finalizados.xlsx pelo site
</commit_message>
<xml_diff>
--- a/jogos/Lista de Jogos Finalizados.xlsx
+++ b/jogos/Lista de Jogos Finalizados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luiz\Desktop\Pasta Geral\0 - Antunes\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1DACB9-14A6-4331-AF6E-0541DD884B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{855241B6-70CF-4C8F-B759-6B616FCDB7E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{185F8663-3FF1-4EF9-AA90-43B25B82DF02}"/>
   </bookViews>
@@ -2956,7 +2956,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2952" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2953" uniqueCount="515">
   <si>
     <t>Nº</t>
   </si>
@@ -5419,6 +5419,21 @@
   </si>
   <si>
     <t>Super Bomberman R</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Super Bomberman R - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>[P]</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -6901,7 +6916,7 @@
         <v>385</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>343</v>
@@ -8255,7 +8270,7 @@
       </c>
       <c r="N25" s="42">
         <f>COUNTIFS(B:B,"*[P]*")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>359</v>
@@ -9008,7 +9023,7 @@
         <v>26</v>
       </c>
       <c r="O39" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M39,1,1), $F:$F, "&lt;="&amp;DATE(M39,12,31))</f>
+        <f t="shared" ref="O39:O51" si="0">SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M39,1,1), $F:$F, "&lt;="&amp;DATE(M39,12,31))</f>
         <v>21.778043981481481</v>
       </c>
       <c r="P39" s="77"/>
@@ -9057,7 +9072,7 @@
         <v>20</v>
       </c>
       <c r="O40" s="78">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M40,1,1), $F:$F, "&lt;="&amp;DATE(M40,12,31))</f>
+        <f t="shared" si="0"/>
         <v>39.712557870370361</v>
       </c>
       <c r="P40" s="79"/>
@@ -9106,7 +9121,7 @@
         <v>24</v>
       </c>
       <c r="O41" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M41,1,1), $F:$F, "&lt;="&amp;DATE(M41,12,31))</f>
+        <f t="shared" si="0"/>
         <v>15.460520833333334</v>
       </c>
       <c r="P41" s="77"/>
@@ -9155,7 +9170,7 @@
         <v>35</v>
       </c>
       <c r="O42" s="78">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M42,1,1), $F:$F, "&lt;="&amp;DATE(M42,12,31))</f>
+        <f t="shared" si="0"/>
         <v>66.78905092592592</v>
       </c>
       <c r="P42" s="79"/>
@@ -9203,7 +9218,7 @@
         <v>33</v>
       </c>
       <c r="O43" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M43,1,1), $F:$F, "&lt;="&amp;DATE(M43,12,31))</f>
+        <f t="shared" si="0"/>
         <v>58.889837962962957</v>
       </c>
       <c r="P43" s="77"/>
@@ -9251,7 +9266,7 @@
         <v>20</v>
       </c>
       <c r="O44" s="78">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M44,1,1), $F:$F, "&lt;="&amp;DATE(M44,12,31))</f>
+        <f t="shared" si="0"/>
         <v>47.408263888888897</v>
       </c>
       <c r="P44" s="79"/>
@@ -9299,7 +9314,7 @@
         <v>29</v>
       </c>
       <c r="O45" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M45,1,1), $F:$F, "&lt;="&amp;DATE(M45,12,31))</f>
+        <f t="shared" si="0"/>
         <v>63.090277777777764</v>
       </c>
       <c r="P45" s="77"/>
@@ -9347,7 +9362,7 @@
         <v>20</v>
       </c>
       <c r="O46" s="78">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M46,1,1), $F:$F, "&lt;="&amp;DATE(M46,12,31))</f>
+        <f t="shared" si="0"/>
         <v>57.896655092592589</v>
       </c>
       <c r="P46" s="79"/>
@@ -9395,7 +9410,7 @@
         <v>50</v>
       </c>
       <c r="O47" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M47,1,1), $F:$F, "&lt;="&amp;DATE(M47,12,31))</f>
+        <f t="shared" si="0"/>
         <v>96.097395833333323</v>
       </c>
       <c r="P47" s="77"/>
@@ -9443,7 +9458,7 @@
         <v>50</v>
       </c>
       <c r="O48" s="78">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M48,1,1), $F:$F, "&lt;="&amp;DATE(M48,12,31))</f>
+        <f t="shared" si="0"/>
         <v>76.722939814814836</v>
       </c>
       <c r="P48" s="79"/>
@@ -9491,7 +9506,7 @@
         <v>20</v>
       </c>
       <c r="O49" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M49,1,1), $F:$F, "&lt;="&amp;DATE(M49,12,31))</f>
+        <f t="shared" si="0"/>
         <v>29.277777777777782</v>
       </c>
       <c r="P49" s="77"/>
@@ -9539,7 +9554,7 @@
         <v>42</v>
       </c>
       <c r="O50" s="78">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M50,1,1), $F:$F, "&lt;="&amp;DATE(M50,12,31))</f>
+        <f t="shared" si="0"/>
         <v>33.481250000000003</v>
       </c>
       <c r="P50" s="79"/>
@@ -9587,7 +9602,7 @@
         <v>16</v>
       </c>
       <c r="O51" s="76">
-        <f>SUMIFS($G:$G, $F:$F, "&gt;="&amp;DATE(M51,1,1), $F:$F, "&lt;="&amp;DATE(M51,12,31))</f>
+        <f t="shared" si="0"/>
         <v>40.547222222222231</v>
       </c>
       <c r="P51" s="77"/>
@@ -21768,22 +21783,22 @@
     <mergeCell ref="O51:P51"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 M24:N34 O26:Q29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576 C3:L1048576">
+  <conditionalFormatting sqref="C1:T2 M3:N22 C3:L1048576 V3:W22 O3:T25 M24:N34 O26:Q29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576">
     <cfRule type="expression" dxfId="24" priority="16">
       <formula>OR(ISNUMBER(FIND("NES",C1)),    ISNUMBER(FIND("SNES",C1)),    ISNUMBER(FIND("N64",C1)),    ISNUMBER(FIND("GC",C1)),    ISNUMBER(FIND("Wii",C1)),    ISNUMBER(FIND("Wii U",C1)),    ISNUMBER(FIND("Switch",C1)),    ISNUMBER(FIND("Switch 2",C1)),    ISNUMBER(FIND("GB",C1)),    ISNUMBER(FIND("GBC",C1)),    ISNUMBER(FIND("GBA",C1)),    ISNUMBER(FIND("DS",C1)),    ISNUMBER(FIND("3DS",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 M24:N34 O26:Q29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576 S26:T29 C3:L1048576">
+  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 C3:L1048576 M24:N34 O26:Q29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576 S26:T29">
     <cfRule type="expression" dxfId="23" priority="18">
       <formula>OR(ISNUMBER(FIND("X One",C1)),    ISNUMBER(FIND("X Series",C1)),    ISNUMBER(FIND("X 360",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 M24:N34 O26:Q29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576 C3:L1048576">
+  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 C3:L1048576 M24:N34 O26:Q29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576">
     <cfRule type="expression" dxfId="22" priority="17">
       <formula>OR(ISNUMBER(FIND("PS1",C1)),    ISNUMBER(FIND("PS2",C1)),    ISNUMBER(FIND("PS3",C1)),    ISNUMBER(FIND("PS4",C1)),    ISNUMBER(FIND("PSP",C1)),    ISNUMBER(FIND("Vita",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 M24:N34 O26:Q29 S26:T29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576 C3:L1048576">
+  <conditionalFormatting sqref="C1:T2 M3:N22 V3:W22 O3:T25 C3:L1048576 M24:N34 O26:Q29 S26:T29 R26:R1048576 O30:O57 M37:N53 S39:T1048576 Q51:Q1048576 M58:P1048576">
     <cfRule type="expression" dxfId="21" priority="19">
       <formula>ISNUMBER(FIND("PC",C1))</formula>
     </cfRule>
@@ -21791,7 +21806,7 @@
       <formula>ISNUMBER(FIND("MD",C1))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M4:M14 H1:H1048576">
+  <conditionalFormatting sqref="H1:H1048576 M4:M14">
     <cfRule type="expression" dxfId="19" priority="11">
       <formula>OR(ISNUMBER(FIND("11",H1)),)</formula>
     </cfRule>
@@ -21813,7 +21828,7 @@
       <formula>NOT(ISERROR(SEARCH("Não",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M1:M22 M24:M34 M37:M53 M58:M1048576 I1:I1048576">
+  <conditionalFormatting sqref="M1:M22 I1:I1048576 M24:M34 M37:M53 M58:M1048576">
     <cfRule type="containsText" dxfId="13" priority="23" operator="containsText" text="Fácil">
       <formula>NOT(ISERROR(SEARCH("Fácil",I1)))</formula>
     </cfRule>
@@ -22488,7 +22503,7 @@
         <v>7</v>
       </c>
       <c r="D18" s="39" t="s">
-        <v>383</v>
+        <v>513</v>
       </c>
       <c r="F18" s="22">
         <v>15</v>
@@ -22526,7 +22541,7 @@
         <v>7</v>
       </c>
       <c r="D19" s="39" t="s">
-        <v>405</v>
+        <v>383</v>
       </c>
       <c r="F19" s="22">
         <v>16</v>
@@ -22564,7 +22579,7 @@
         <v>7</v>
       </c>
       <c r="D20" s="39" t="s">
-        <v>509</v>
+        <v>405</v>
       </c>
       <c r="F20" s="22">
         <v>17</v>
@@ -22602,7 +22617,7 @@
         <v>7</v>
       </c>
       <c r="D21" s="39" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F21" s="22">
         <v>18</v>
@@ -22640,7 +22655,7 @@
         <v>7</v>
       </c>
       <c r="D22" s="39" t="s">
-        <v>406</v>
+        <v>510</v>
       </c>
       <c r="F22" s="22">
         <v>19</v>
@@ -22675,10 +22690,10 @@
         <v>20</v>
       </c>
       <c r="C23" s="21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D23" s="39" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
       <c r="F23" s="22">
         <v>20</v>
@@ -22716,7 +22731,7 @@
         <v>6</v>
       </c>
       <c r="D24" s="39" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="J24" s="22">
         <v>21</v>
@@ -22745,7 +22760,7 @@
         <v>6</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="J25" s="22">
         <v>22</v>
@@ -22774,7 +22789,7 @@
         <v>6</v>
       </c>
       <c r="D26" s="39" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J26" s="22">
         <v>23</v>
@@ -22803,7 +22818,7 @@
         <v>6</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>508</v>
+        <v>386</v>
       </c>
       <c r="J27" s="22">
         <v>24</v>
@@ -22832,7 +22847,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>380</v>
+        <v>508</v>
       </c>
       <c r="N28" s="22">
         <v>25</v>
@@ -22845,6 +22860,15 @@
       </c>
     </row>
     <row r="29" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B29" s="22">
+        <v>26</v>
+      </c>
+      <c r="C29" s="21">
+        <v>6</v>
+      </c>
+      <c r="D29" s="39" t="s">
+        <v>380</v>
+      </c>
       <c r="N29" s="22">
         <v>26</v>
       </c>

</xml_diff>